<commit_message>
spec: retire supports-goals and fulfills-requirements; fix 18 four-part relationship ids
supports-goals and fulfills-requirements were traceability-category twins of
supports and fulfills with the same meaning and the same inverse, which the
charter forbids. The nine testing-layer schemas that used them now use the
surviving predicate; both are removed from predicates.json (69 predicates).
applied-synonyms.json records the two predicate retirements and nine renames
for the dr upgrade migration; the migration table is regenerated (126 triple
rules, 3 predicate renames). The four testing rows of the walk sheet and the
reflection plan that named the old triples are renamed with them.

18 relationship schemas had a four-part id with no destination-layer segment
(e.g. security.securitymodel.aggregates.role); every id is now the five-part
form. No other field changed and no model migration is needed.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cli/scripts/spec-enrich/data/triage/reflect/clef/walk-sheet.xlsx
+++ b/cli/scripts/spec-enrich/data/triage/reflect/clef/walk-sheet.xlsx
@@ -10751,7 +10751,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>testing.testcasesketch.supports-goals.motivation.goal</t>
+          <t>testing.testcasesketch.supports.motivation.goal</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -10796,7 +10796,7 @@
       </c>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>testing.testcoveragemodel.supports-goals.motivation.goal (exists)</t>
+          <t>testing.testcoveragemodel.supports.motivation.goal (exists)</t>
         </is>
       </c>
       <c r="N41" s="2" t="inlineStr">
@@ -10806,13 +10806,13 @@
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>to testing.testcoveragemodel.supports-goals.motivation.goal (a migration drops the old edge)</t>
+          <t>to testing.testcoveragemodel.supports.motivation.goal (a migration drops the old edge)</t>
         </is>
       </c>
       <c r="P41" s="4" t="n"/>
       <c r="Q41" s="4" t="inlineStr">
         <is>
-          <t>testing.testcoveragemodel.supports-goals.motivation.goal</t>
+          <t>testing.testcoveragemodel.supports.motivation.goal</t>
         </is>
       </c>
       <c r="R41" s="4" t="n"/>
@@ -10913,7 +10913,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>testing.testcoveragetarget.supports-goals.motivation.goal</t>
+          <t>testing.testcoveragetarget.supports.motivation.goal</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -10958,7 +10958,7 @@
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>testing.testcoveragemodel.supports-goals.motivation.goal (exists)</t>
+          <t>testing.testcoveragemodel.supports.motivation.goal (exists)</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
@@ -10968,13 +10968,13 @@
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>to testing.testcoveragemodel.supports-goals.motivation.goal (a migration drops the old edge)</t>
+          <t>to testing.testcoveragemodel.supports.motivation.goal (a migration drops the old edge)</t>
         </is>
       </c>
       <c r="P43" s="4" t="n"/>
       <c r="Q43" s="4" t="inlineStr">
         <is>
-          <t>testing.testcoveragemodel.supports-goals.motivation.goal</t>
+          <t>testing.testcoveragemodel.supports.motivation.goal</t>
         </is>
       </c>
       <c r="R43" s="4" t="n"/>
@@ -11158,7 +11158,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>testing.testcoveragetarget.fulfills-requirements.motivation.requirement</t>
+          <t>testing.testcoveragetarget.fulfills.motivation.requirement</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -11401,7 +11401,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>testing.testcoveragemodel.fulfills-requirements.motivation.requirement</t>
+          <t>testing.testcoveragemodel.fulfills.motivation.requirement</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">

</xml_diff>